<commit_message>
Add demo code, ignore large video file
</commit_message>
<xml_diff>
--- a/scenarios.xlsx
+++ b/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francescocompagno/Desktop/Work_Units/Codebases_to_publish/ESWC_2026_Demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF025235-A53A-A148-BFDB-6524F758B4D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FD5C58-66BA-7C47-BCBD-6153B5180BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{FC7576A7-5561-E04F-B1AC-279C300660B2}"/>
+    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" xr2:uid="{FC7576A7-5561-E04F-B1AC-279C300660B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="94">
   <si>
     <t>Scenario</t>
   </si>
@@ -261,9 +261,6 @@
     <t>cable detached from switch in control x</t>
   </si>
   <si>
-    <t>The led of all the control modules are missing</t>
-  </si>
-  <si>
     <t xml:space="preserve">One of the 8 switches modules is detatched from one of the corresponding cables. To make testing more challenging all the control module leds have been removed. Fastest way to diagnose is to use the power supply led to bisect-testing the control modules. </t>
   </si>
   <si>
@@ -313,6 +310,15 @@
   </si>
   <si>
     <t xml:space="preserve">  -&gt; Clarify and observe the actual symptoms presented by the system, since the listed symptoms ([omissis]) do not specify any observable issue.</t>
+  </si>
+  <si>
+    <t>The led on the power supply module is on</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All the leds on the control modules are missing </t>
+  </si>
+  <si>
+    <t>The lamp does not turn on when a battery is inserted in the circuit and all the switches are in the on position</t>
   </si>
 </sst>
 </file>
@@ -698,7 +704,7 @@
     <col min="1" max="1" width="24.1640625" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" customWidth="1"/>
     <col min="3" max="3" width="72" customWidth="1"/>
-    <col min="4" max="4" width="74.33203125" customWidth="1"/>
+    <col min="4" max="4" width="88.1640625" customWidth="1"/>
     <col min="5" max="5" width="46" customWidth="1"/>
     <col min="6" max="6" width="36.5" customWidth="1"/>
     <col min="7" max="7" width="41.33203125" customWidth="1"/>
@@ -874,10 +880,10 @@
         <v>59</v>
       </c>
       <c r="B26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" t="s">
         <v>83</v>
-      </c>
-      <c r="C26" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -885,10 +891,10 @@
         <v>72</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -899,20 +905,20 @@
         <v>73</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D34" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D35" t="s">
-        <v>53</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -920,10 +926,10 @@
         <v>72</v>
       </c>
       <c r="B38" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" t="s">
         <v>85</v>
-      </c>
-      <c r="C38" t="s">
-        <v>86</v>
       </c>
       <c r="D38" t="s">
         <v>52</v>
@@ -936,32 +942,32 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>77</v>
+      </c>
+      <c r="B42" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" t="s">
         <v>78</v>
-      </c>
-      <c r="B42" t="s">
-        <v>77</v>
-      </c>
-      <c r="C42" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B46" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" t="s">
         <v>80</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>81</v>
-      </c>
-      <c r="D46" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
@@ -1034,7 +1040,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -1356,7 +1362,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="H42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -1370,7 +1376,7 @@
         <v>17</v>
       </c>
       <c r="H43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -1381,7 +1387,7 @@
         <v>54</v>
       </c>
       <c r="H44" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Corrected various bugs in the symbolic assistant. Various betterments. Discontinued xslx with a csv. Various testing.
</commit_message>
<xml_diff>
--- a/scenarios.xlsx
+++ b/scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francescocompagno/Desktop/Work_Units/Codebases_to_publish/ESWC_2026_Demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FD5C58-66BA-7C47-BCBD-6153B5180BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCDB2889-C802-BD46-8847-E9B90184C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" xr2:uid="{FC7576A7-5561-E04F-B1AC-279C300660B2}"/>
+    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{FC7576A7-5561-E04F-B1AC-279C300660B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="102">
   <si>
     <t>Scenario</t>
   </si>
@@ -192,9 +192,6 @@
     <t>this one was with 1 symptom: "lamp does not turn no" -&gt; {'Switch', 'Cables', 'Battery', 'MainLoad'}</t>
   </si>
   <si>
-    <t>10 cubes - detached switch in control 2</t>
-  </si>
-  <si>
     <t>The lamp does not turn on when all the switches are in the on position (that is, they are closed)</t>
   </si>
   <si>
@@ -319,6 +316,33 @@
   </si>
   <si>
     <t>The lamp does not turn on when a battery is inserted in the circuit and all the switches are in the on position</t>
+  </si>
+  <si>
+    <t>LLM Second guesses input</t>
+  </si>
+  <si>
+    <t>10 cubes - detached switch in control x</t>
+  </si>
+  <si>
+    <t>detached switch in control 3</t>
+  </si>
+  <si>
+    <t>DIAGNOSTIC_SCENARIO_RUN_2026-03-02T19:11:06</t>
+  </si>
+  <si>
+    <t>It works as intended: first some cheap tests are explored, then bisection strategy</t>
+  </si>
+  <si>
+    <t>1, 3, 3, 3(*7)</t>
+  </si>
+  <si>
+    <t>1, 3, 3, 3, 3, 3, 3, 3, 3, 3, 3</t>
+  </si>
+  <si>
+    <t>Example of sequential search</t>
+  </si>
+  <si>
+    <t>Last one is actually 3*7 = 21… It proposes sequential search strategy, plus is inconsistent on the instruction structure</t>
   </si>
 </sst>
 </file>
@@ -716,27 +740,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" t="s">
         <v>56</v>
-      </c>
-      <c r="C1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
         <v>59</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>61</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
@@ -754,13 +778,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" t="s">
         <v>62</v>
-      </c>
-      <c r="C6" t="s">
-        <v>63</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -781,13 +805,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" t="s">
-        <v>65</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -805,13 +829,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" t="s">
         <v>66</v>
-      </c>
-      <c r="C14" t="s">
-        <v>67</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -829,13 +853,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" t="s">
         <v>68</v>
-      </c>
-      <c r="C18" t="s">
-        <v>69</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -853,13 +877,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" t="s">
         <v>70</v>
-      </c>
-      <c r="C22" t="s">
-        <v>71</v>
       </c>
       <c r="D22" t="s">
         <v>5</v>
@@ -877,97 +901,97 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" t="s">
         <v>82</v>
-      </c>
-      <c r="C26" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" t="s">
         <v>72</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>73</v>
       </c>
-      <c r="C34" t="s">
-        <v>74</v>
-      </c>
       <c r="D34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" t="s">
         <v>84</v>
       </c>
-      <c r="C38" t="s">
-        <v>85</v>
-      </c>
       <c r="D38" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D40" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" t="s">
         <v>77</v>
-      </c>
-      <c r="B42" t="s">
-        <v>76</v>
-      </c>
-      <c r="C42" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B46" t="s">
+        <v>78</v>
+      </c>
+      <c r="C46" t="s">
         <v>79</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>80</v>
-      </c>
-      <c r="D46" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
@@ -987,7 +1011,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C46E0770-1A43-B449-8786-4030E834DA3B}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="74.33203125" customWidth="1"/>
@@ -1040,7 +1064,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H2" t="s">
         <v>9</v>
@@ -1362,51 +1386,119 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="H42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" t="s">
         <v>51</v>
-      </c>
-      <c r="B43" t="s">
-        <v>52</v>
       </c>
       <c r="C43" t="s">
         <v>17</v>
       </c>
       <c r="H43" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" t="s">
         <v>53</v>
       </c>
-      <c r="C44" t="s">
-        <v>54</v>
-      </c>
       <c r="H44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C45" t="s">
         <v>19</v>
       </c>
+      <c r="H45" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C48" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>90</v>
+      </c>
+      <c r="C50" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" t="s">
+        <v>33</v>
+      </c>
+      <c r="E50" t="s">
+        <v>96</v>
+      </c>
+      <c r="F50" t="s">
+        <v>97</v>
+      </c>
+      <c r="G50" t="s">
+        <v>99</v>
+      </c>
+      <c r="H50" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>91</v>
+      </c>
+      <c r="C51" t="s">
+        <v>95</v>
+      </c>
+      <c r="G51" t="s">
+        <v>98</v>
+      </c>
+      <c r="H51" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B52" t="s">
+        <v>92</v>
+      </c>
+      <c r="C52" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C53" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C54" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C55" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C56" s="1" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Run a few experiments and adjusted code accordingly
</commit_message>
<xml_diff>
--- a/scenarios.xlsx
+++ b/scenarios.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francescocompagno/Desktop/Work_Units/Codebases_to_publish/ESWC_2026_Demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCDB2889-C802-BD46-8847-E9B90184C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35A89E21-5E40-A041-92DE-D76A6387CD22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{FC7576A7-5561-E04F-B1AC-279C300660B2}"/>
+    <workbookView xWindow="14160" yWindow="1080" windowWidth="27640" windowHeight="16940" xr2:uid="{FC7576A7-5561-E04F-B1AC-279C300660B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenarios" sheetId="2" r:id="rId1"/>
     <sheet name="Notes about scenarios" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1018,7 +1019,7 @@
     <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="36.5" customWidth="1"/>
     <col min="5" max="5" width="41.33203125" customWidth="1"/>
-    <col min="6" max="6" width="65.33203125" customWidth="1"/>
+    <col min="6" max="6" width="17.1640625" customWidth="1"/>
     <col min="7" max="7" width="24.1640625" customWidth="1"/>
     <col min="8" max="8" width="25.6640625" customWidth="1"/>
     <col min="9" max="9" width="19.5" customWidth="1"/>

</xml_diff>